<commit_message>
Agregar las métricas del núcleo y la lista de pendientes
- eval/metricas.py: cobertura de citas, eficiencia, tokens y costo; con la planilla
  etiquetada, macro-F1 de temas (LLM vs embeddings vs palabras clave), relación con Panamá,
  Precision@k, precisión y recall de la agrupación, validez de sustento y kappa
- Planilla ampliada con las hojas Agenda, Pares y Afirmaciones (Etiquetas sin cambios)
- PENDIENTES.md con la validación de consultas con preguntas nuevas y lo que falta
</commit_message>
<xml_diff>
--- a/backend/eval/planilla_etiquetas.xlsx
+++ b/backend/eval/planilla_etiquetas.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Etiquetas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Agenda" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Pares" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Afirmaciones" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -448,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -467,163 +470,166 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Para qué sirve: medir con datos reales si el sistema clasifica bien. Sus respuestas son la referencia contra la que se compara el LLM.</t>
+          <t>Para qué sirve: medir con datos reales si el sistema acierta. Sus respuestas son la referencia contra la que se compara. Complete las columnas amarillas con los menús desplegables. Si etiquetan dos personas, cada una usa su propia copia del archivo y no se consultan entre sí.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Cómo completarla:</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>1. Lea solo el titular (no busque la nota): el sistema tampoco ve más que eso.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Hoja Etiquetas (100 titulares)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. En la hoja Etiquetas complete las columnas amarillas usando los menús desplegables.</t>
+          <t>Lea solo el titular (no busque la nota): el sistema tampoco ve más que eso. No consulte las respuestas del sistema. Si duda entre un tema y "otro", elija "otro" y explique en notas.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>3. No consulte las respuestas del sistema antes de terminar.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Columna tema:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>4. Si duda entre un tema y "otro", elija "otro" y explique en notas.</t>
+          <t xml:space="preserve">  economia: inflación, precios, crecimiento, empleo y desempleo, deuda, impuestos, finanzas públicas, inversión y comercio. NO: consejos de finanzas personales.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>5. Si etiquetan dos personas, cada una usa su propia copia del archivo.</t>
+          <t xml:space="preserve">  logistica_canal: Canal de Panamá, buques, puertos, contenedores, comercio exterior y cadena logística. NO: sanciones o conflictos de otros países sin efecto en esa logística.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  turismo: turistas, hoteles, vuelos, aerolíneas, cruceros y actividad turística.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Columna tema</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  servicios_publicos: servicios que presta el Estado: agua potable, electricidad, transporte público, metro, carreteras, recolección de basura, hospitales públicos, CSS y campañas del Ministerio de Salud. NO: consejos de salud personal, testimonios o historias de vida, farándula, ni sucesos policiales.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  economia: inflación, precios, crecimiento, empleo y desempleo, deuda, impuestos, finanzas públicas, inversión y comercio. NO: consejos de finanzas personales.</t>
+          <t xml:space="preserve">  eventos_naturales: sismos, lluvias, inundaciones, sequías, deslizamientos, fenómenos climáticos y simulacros o alertas ante ellos.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  logistica_canal: Canal de Panamá, buques, puertos, contenedores, comercio exterior y cadena logística. NO: sanciones o conflictos de otros países sin efecto en esa logística.</t>
+          <t xml:space="preserve">  regulacion: leyes, decretos, normas, acuerdos de superintendencias y fallos judiciales de Panamá. NO: procesos judiciales de otros países.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  turismo: turistas, hoteles, vuelos, aerolíneas, cruceros y actividad turística.</t>
+          <t xml:space="preserve">  otro: lo que no encaja claramente en los anteriores: deportes, farándula, entretenimiento, salud y bienestar personal, sucesos policiales, política o justicia de otros países.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  servicios_publicos: servicios que presta el Estado: agua potable, electricidad, transporte público, metro, carreteras, recolección de basura, hospitales públicos, CSS y campañas del Ministerio de Salud. NO: consejos de salud personal, testimonios o historias de vida, farándula, ni sucesos policiales.</t>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Columna relacion_panama:</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  eventos_naturales: sismos, lluvias, inundaciones, sequías, deslizamientos, fenómenos climáticos y simulacros o alertas ante ellos.</t>
+          <t xml:space="preserve">  directa: ocurre en Panamá o involucra directamente a instituciones, personas o empresas de Panamá</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  regulacion: leyes, decretos, normas, acuerdos de superintendencias y fallos judiciales de Panamá. NO: procesos judiciales de otros países.</t>
+          <t xml:space="preserve">  indirecta: ocurre fuera, pero tiene un efecto concreto y explicable en Panamá (ej. comercio, Canal, migración)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  otro: lo que no encaja claramente en los anteriores: deportes, farándula, entretenimiento, salud y bienestar personal, sucesos policiales, política o justicia de otros países.</t>
+          <t xml:space="preserve">  ninguna: no ocurre en Panamá ni tiene un efecto concreto en Panamá</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Columna en_agenda_tvn: "si" si un editor de TVN debería considerarla para la agenda del día; "no" si no merece revisión editorial hoy.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Columna relacion_panama</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  directa: ocurre en Panamá o involucra directamente a instituciones, personas o empresas de Panamá</t>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Hoja Agenda (15 eventos)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  indirecta: ocurre fuera, pero tiene un efecto concreto y explicable en Panamá (ej. comercio, Canal, migración)</t>
+          <t>Son los casos que el sistema puso arriba, en un orden mezclado a propósito. Para cada uno: ¿un editor de TVN debería considerarlo para la agenda del día? (si / no).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ninguna: no ocurre en Panamá ni tiene un efecto concreto en Panamá</t>
-        </is>
-      </c>
+      <c r="A23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Hoja Pares (40 pares de titulares)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Columna en_agenda_tvn</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>¿Los dos titulares hablan del MISMO hecho concreto (no solo del mismo tema)? Ejemplo: dos notas sobre el mismo sismo = si; una sobre un sismo y otra sobre otro sismo = no.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  si: un editor de TVN debería considerarla para la agenda del día.</t>
-        </is>
-      </c>
+      <c r="A26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  no: no merece revisión editorial hoy (irrelevante, de nicho, entretenimiento...).</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Hoja Afirmaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Aquí sí se muestra lo que escribió el sistema, junto con lo que cita. Juzgue SOLO si lo citado respalda la afirmación: si = la respalda completa; parcial = respalda una parte o exagera; no = no la respalda o agrega algo que no está en lo citado.</t>
         </is>
       </c>
     </row>
@@ -3613,4 +3619,2526 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id_evento</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>titulo</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>medios</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>noticias</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>en_agenda_tvn</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-e7673d45b48a</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Lau Cortés: Ordenan detención domiciliaria e imputan cargos por enriquecimiento injustificado y blanqueo de capitales</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-2a41592af821</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Ifarhu fija hasta el 14 de octubre para entregar boletín de Becas de Excelencia</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-e2e7ae51395c</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>ITSE se suma a iniciativa para proyectar el café panameño y formar baristas</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-d6b4d86d3dcb</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Exportaciones de banano superan los $17 millones en junio y marcan recuperación</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-64a1fae98dc4</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>EEUU intercepta 90 embarques de combustible a Cuba</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-1a8d986bf866</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-33f2663b5f67</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>MOP avanza en mas del 45% nueva ruta para desahogar la via Interamericana en David</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-5bf4576df900</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Asamblea: Debate por la renovación del contrato de Ciudad del Saber genera cuestionamientos por exoneraciones</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-7f5a31e89279</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Bocas del Toro afina detalles para el III Simulacro de Evacuación este lunes 12 de octubre</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-c4339fd4cfad</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Descuentos para jubilados: Proyecto modificado plantea 30% menos en compra de pañales, telefonía y otros beneficios</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-4b2fc0678f6c</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Panamá y OIM evalúan trasladar de Costa Rica a Panamá una oficina de coordinación migratoria</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-3d58bd578f4b</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>EV-N-009b376481c1</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Idaan amplía proyectos de agua potable en Changuinola y otros puntos de Bocas del Toro</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una opción del menú desplegable." type="list">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id_a</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>titulo_a</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>medio_a</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>id_b</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>titulo_b</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>medio_b</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
+          <t>mismo_evento</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>N-bb6623b6bdee</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Navidad 2026 de la Alcaldía de Panamá superaría los $3. 8 millones en contratos</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>midiario.com</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>N-3a7287fdd261</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Terminal 3 de Tocumen: un proyecto de $3, 500 millones que Panamá aún no necesita</t>
+        </is>
+      </c>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>N-1af6371f378c</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Lluvias y tormentas esta tarde: ¿Dónde se concentrarán los aguaceros más fuertes?</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>telemetro.com</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>N-3caa90ccd905</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Paraguas a mano: lluvias y tormentas seguirán hasta el sábado</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>prensa.com</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="n"/>
+      <c r="I3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>N-18fb2324db75</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>La sociedad que estamos formando</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>prensa.com</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>N-c0c3e5bd15ab</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Hacer la diferencia en un mundo cambiante</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>prensa.com</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>N-c53d81bbfc62</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Rosh Hashaná 2026: ¿quiénes tendrán libre este sábado 12 de septiembre en Panamá por el Año Nuevo judío?</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>telemetro.com</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>N-ad5299e55159</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Qué beneficio gratis tienen colombianos en viaje a Panamá desde septiembre 2026</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>pulzo.com</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>N-5f960815999a</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Panamá sigue moviendo sus fichas para atraer inversiones y fortalecer sus relaciones con Emiratos Árabes Unidos</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>N-7a752b31c5cd</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Panamá se consolida como uno de los mercados de entretenimiento digital de Centroamérica</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>nuevaya.com.ni</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>N-6569c9fb0568</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>D - Max, el prófugo colombiano que estuvo encarcelado en Panamá bajo un nombre falso</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>N-2017f1b96d8a</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Miembro de red de sicarios buscado en Colombia estuvo preso en Panamá bajo un nombre falso</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>N-5f960815999a</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Panamá sigue moviendo sus fichas para atraer inversiones y fortalecer sus relaciones con Emiratos Árabes Unidos</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>N-bc1ff42d5c5b</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Panamá y Filipinas fortalecen cooperación mediante nuevo mecanismo de consultas políticas – Ministerio de Relaciones exteriores</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>mire.gob.pa</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="n"/>
+      <c r="I8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>N-b1a3f3391951</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>ONG fantasma e instigación al vandalismo, los señalamientos sobre los policías encubiertos</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>N-7b739feeade0</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Panamá: policía admite agentes encubiertos en organizaciones sociales</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>telesurtv.net</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>N-216df2f64f80</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Panamá confía en salir de la lista fiscal de la Unión Europea en octubre</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>N-5f960815999a</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Panamá sigue moviendo sus fichas para atraer inversiones y fortalecer sus relaciones con Emiratos Árabes Unidos</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="n"/>
+      <c r="I10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>N-585dbcd0c409</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>José Emilio Moreno asume la rectoría de la UP y anuncia una nueva carrera</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>telemetro.com</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>N-6ccfebe68382</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Mármol, Honoris Causa – Universidad APEC, plantea usar educación, inteligencia artificial y poesía para defender al ser humano</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>acento.com.do</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="n"/>
+      <c r="I11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>N-729987434438</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media y Capadeso sellan alianza para visibilizar labor social</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>N-c9c0832cfa23</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media y Fundamorgan firman alianza para sensibilizar sobre la problemáticas sociales como la violencia</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="n"/>
+      <c r="I12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>N-bbb6b0847738</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Niños y adolescentes hospitalizados podrán continuar sus estudios con aulas de atención hospitalaria</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>N-14447c0d5d2e</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>Meduca y CSS firman acuerdo para el programa de Aulas de Atención Hospitalaria</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>telemetro.com</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="n"/>
+      <c r="I13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>N-4e8be96ab6f5</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>MLB Playoffs 2026 resultado| Cerveceros dejan fuera a Padres y van por el banderín de la Liga Nacional ante Dodgers</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>N-4ba0d048d89d</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>MLB Playoffs 2026 resultado| Guardianes, con el panameño Daniel Espino como abridor, se revitalizan ante Medias Blancas en la Serie Divisional</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="H14" s="7" t="n"/>
+      <c r="I14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>N-6f0f5de359ff</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Panamá y New York Institute of Technology exploran alianza de cooperación académica, científica y tecnológica – Ministerio de Relaciones exteriores</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>mire.gob.pa</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>N-bc1ff42d5c5b</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Panamá y Filipinas fortalecen cooperación mediante nuevo mecanismo de consultas políticas – Ministerio de Relaciones exteriores</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>mire.gob.pa</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="n"/>
+      <c r="I15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>N-0803c58d1f47</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media recibe reconocimiento en el Simposio Internacional de Innovación en Sostenibilidad: Edificio y Ciudad</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>N-b8c36c576356</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media dice presente en la Teletón 20-30 con una donación de 100,000 dólares</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="H16" s="7" t="n"/>
+      <c r="I16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>N-40e03a36285a</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Presupuesto del Canal fue aprobado en tercer debate</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>N-18b69feaf74f</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Canal de Panamá manejará presupuesto de B /. 5, 555 millones para 2027</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>critica.com.pa</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="n"/>
+      <c r="I17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>N-5f960815999a</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>Panamá sigue moviendo sus fichas para atraer inversiones y fortalecer sus relaciones con Emiratos Árabes Unidos</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>N-8fe9c7059ab0</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Cinco grandes bancos e inversionistas muestran apetito por Panamá</t>
+        </is>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="H18" s="7" t="n"/>
+      <c r="I18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>N-6f0f5de359ff</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Panamá y New York Institute of Technology exploran alianza de cooperación académica, científica y tecnológica – Ministerio de Relaciones exteriores</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>mire.gob.pa</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>N-7bd9d18569c3</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Panamá propone una cooperación iberoamericana orientada a resultados y la defensa de la democracia y los derechos políticos – Ministerio de Relaciones exteriores</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>mire.gob.pa</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="n"/>
+      <c r="I19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>N-75d30d184a8e</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Vacaciones escolares: el descanso que protege la salud mental de los niños</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>N-47f8ee7205c7</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Vacaciones escolares: el descanso que protege la salud mental de los niños</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="H20" s="7" t="n"/>
+      <c r="I20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>N-f3551b42978b</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Panamá enfrenta reto de agilizar movimiento de carga frente a sus competidores</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>N-07a6a4238cdc</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Falta de contundencia ante Nueva Zelanda evidencia el gran dilema ofensivo de Panamá</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="n"/>
+      <c r="I21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>N-07a6a4238cdc</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Falta de contundencia ante Nueva Zelanda evidencia el gran dilema ofensivo de Panamá</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>laestrella.com.pa</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>N-26cefa4637f9</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Christiansen explica las carencias de Panamá ante Nueva Zelanda</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="H22" s="7" t="n"/>
+      <c r="I22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>N-4844a941084a</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media y Sabores de Colón se unen para resaltar la gastronomía y cultura colonense</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>N-438971e86c21</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Una alianza por el conocimiento: Ciudad del Saber y TVN Media unen esfuerzos</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="n"/>
+      <c r="I23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>N-bf599988a47d</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media presenta su Informe de Sostenibilidad bajo los principios de Ambiente, Sociedad y Gobernanza</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>N-dd32c6a3ff45</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>TVN Media recibe reconocimiento por su compromiso ambiental en el programa 'Reduce Tu Huella'</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>TVN</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="n"/>
+      <c r="I24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>N-6276aeb0b476</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>No defendemos cargo: Balbina Herrera reta a la bancada del PRD por la reforma que le da más poder a Benicio Robinson</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>prensa.com</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>N-e4e6f5213d0b</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Balbina Herrera Rejects Changes that would Concentrate the PRD Legal Representation in the Party Presidency.</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>newsroompanama.com</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>N-f459fe75d799</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Preview - Asamblea de Panamá</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>asamblea.gob.pa</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>N-acda0e91bd04</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Preview - Asamblea de Panamá</t>
+        </is>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>asamblea.gob.pa</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="n"/>
+      <c r="I26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>N-095a7b080989</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Localizan los cuerpos de dos rescatistas tras emergencia en el Can de Macho de Monte en Chiriqu</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>N-1b60c24cbe00</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Los riesgos del deber: Mulino lamenta muerte de rescatistas en Macho de Monte</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>telemetro.com</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="n"/>
+      <c r="I27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>N-dbff424687fd</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Hoy Tamaulipas - Tamaulipas Erasmo Gonzalez Robledo rinde su Segundo Informe de Gobierno</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>hoytamaulipas.net</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>N-95b5bc6945da</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="inlineStr">
+        <is>
+          <t>Erasmo González Robledo rinde Segundo Informe de Gobierno</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>horacero.com.mx</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="n"/>
+      <c r="I28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>N-f3551b42978b</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Panamá enfrenta reto de agilizar movimiento de carga frente a sus competidores</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>panamaamerica.com.pa</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>N-5f960815999a</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Panamá sigue moviendo sus fichas para atraer inversiones y fortalecer sus relaciones con Emiratos Árabes Unidos</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>diaadia.com.pa</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="n"/>
+      <c r="I29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>N-94f1bec3106d</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Ecuador pierde en los penaltis ante Japón y se medirá a Panamá</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>prensa.com</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>N-05b438df49e4</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>La Selección de Panamá ya llegó a Japón para próximos compromisos</t>
+        </is>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>rpctv.com</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="n"/>
+      <c r="I30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>N-97e773785a2f</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>JEP bajo la lupa por arriendo de su sede en Torre Squadra</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>lafm.com.co</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>N-9d6e812d8f9f</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>Revelan los millonarios gastos de la JEP: arriendo, eventos y viajes a Miami</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>lafm.com.co</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="n"/>
+      <c r="I31" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una opción del menú desplegable." type="list">
+      <formula1>"si,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>id_caso</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>origen</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>lo_que_cita</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>respaldada</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Mitradel publico nuevas vacantes de empleo en su portal, segun reporto TVN el 7 de octubre de 2026.</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"
+[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="n"/>
+      <c r="G2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (hecho)</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>La tasa de desempleo anual en Panama para el ano 2024 fue de 8.451% de la poblacion activa.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (hecho)</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>En 2023, la tasa de desempleo registrada en Panama fue de 6.544%.</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="7" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>brief</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>El medio TVN publico el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] que Mitradel habilito nuevas vacantes de empleo en su portal web [N-6ffd1c40b65f:titulo].</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>brief</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Por otro lado, los datos historicos del Banco Mundial indican que en el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] la tasa de desempleo en Panama fue de 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa, mostrando un incremento en comparacion con el 6.544% [WB:PAN:SL.UEM.TOTL.ZS:2024:serie] registrado en el ano 2023 [WB:PAN:SL.UEM.TOTL.ZS:2024:serie].</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]
+[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>brief</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>En la region, para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio], Costa Rica registro 6.936% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] y Republica Dominicana 5.312% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion].</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]
+[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>El medio TVN informo el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] sobre la publicacion de nuevas vacantes de empleo en el portal de Mitradel [N-6ffd1c40b65f:titulo].</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Esta iniciativa surge en un contexto donde, segun datos historicos del Banco Mundial, la tasa de desempleo en Panama para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] se situo en 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa.</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Esta cifra represento un aumento frente al 6.544% [WB:PAN:SL.UEM.TOTL.ZS:2024:serie] reportado en el ano 2023 [WB:PAN:SL.UEM.TOTL.ZS:2024:serie].</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]
+[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>En la comparacion regional del ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio], Costa Rica registro un desempleo de 6.936% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] y Republica Dominicana un 5.312% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion].</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]
+[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>copy_digital</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Mitradel publica nuevas vacantes de empleo en su portal web, segun reporto TVN el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] [N-6ffd1c40b65f:titulo].</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-6ffd1c40b65f</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>copy_digital</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Como contexto historico, la tasa de desempleo en Panama para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] fue de 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa, segun registros del Banco Mundial [WB:PAN:SL.UEM.TOTL.ZS:2024:valor].</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-3d58bd578f4b</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Según un titular publicado por el medio TVN el 8 de octubre de 2026, más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>[N-3d58bd578f4b:titulo] "Más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas"
+[N-3d58bd578f4b:fecha] "2026-10-08T18:27:29Z"</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-33f2663b5f67</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>El titular informa que el MOP avanza en más del 45% una nueva ruta para desahogar la vía Interamericana en David.</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>[N-33f2663b5f67:titulo] "MOP avanza en mas del 45% nueva ruta para desahogar la via Interamericana en David"</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-7f5a31e89279</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>TVN reporta que en Bocas del Toro se están afinando los detalles para el III Simulacro de Evacuación.</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>[N-7f5a31e89279:titulo] "Bocas del Toro afina detalles para el III Simulacro de Evacuación este lunes 12 de octubre"</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-7f5a31e89279</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>El simulacro está programado para el lunes 12 de octubre.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>[N-7f5a31e89279:titulo] "Bocas del Toro afina detalles para el III Simulacro de Evacuación este lunes 12 de octubre"</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n"/>
+      <c r="G17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-c4339fd4cfad</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>El proyecto modificado plantea 30% menos en compra de pañales, telefonía y otros beneficios para jubilados.</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>[N-c4339fd4cfad:titulo] "Descuentos para jubilados: Proyecto modificado plantea 30% menos en compra de pañales, telefonía y otros beneficios"</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-1a8d986bf866</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>[N-1a8d986bf866:titulo] "Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público"</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-e2e7ae51395c</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>El ITSE se incorpora a una iniciativa que busca proyectar el café panameño y capacitar baristas.</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>[N-e2e7ae51395c:titulo] "ITSE se suma a iniciativa para proyectar el café panameño y formar baristas"</t>
+        </is>
+      </c>
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>TVN publicó un titular que indica que el FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026.</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-34877dd09e6b:medio] "TVN"</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>TVN publicó un titular que pregunta si subirán las cuotas de préstamos y menciona que un economista explica el impacto de las tasas de interés en la economía panameña.</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"
+[N-bc0c4a46f2c5:medio] "TVN"</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>brief</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>TVN publicó un titular indicando que el FMI proyecta un crecimiento cercano al 5% para la economía de Panamá en 2026 [N-34877dd09e6b:titulo].</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>brief</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>En otra publicación, el medio plantea la pregunta sobre si subirán las cuotas de préstamos, citando a un economista que explica el impacto de las tasas de interés [N-bc0c4a46f2c5:titulo].</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>El primero indica que el FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026 [N-34877dd09e6b:titulo].</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Esta información fue publicada por el medio el 7 de octubre de 2026 [N-34877dd09e6b:fecha].</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>[N-34877dd09e6b:fecha] "2026-10-07T22:00:00Z"</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>En una segunda nota, TVN pregunta si subirán las cuotas de préstamos, mencionando que un economista explica el impacto de las tasas de interés en la economía panameña [N-bc0c4a46f2c5:titulo].</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>guion_45_60s</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Esta publicación data del 8 de octubre de 2026 [N-bc0c4a46f2c5:fecha].</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>[N-bc0c4a46f2c5:fecha] "2026-10-08T13:23:50Z"</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-34877dd09e6b</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>copy_digital</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>TVN reporta que el FMI proyecta un crecimiento cercano al 5% para 2026 [N-34877dd09e6b:titulo] y debate el impacto de las tasas de interés en las cuotas de préstamos [N-bc0c4a46f2c5:titulo].</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-e7673d45b48a</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>TVN informa que se ordenó la detención domiciliaria e imputaron cargos a Lau Cortés por enriquecimiento injustificado y blanqueo de capitales.</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>[N-e7673d45b48a:titulo] "Lau Cortés: Ordenan detención domiciliaria e imputan cargos por enriquecimiento injustificado y blanqueo de capitales"</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>CASO-EV-N-5bf4576df900</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>afirmación (declaracion)</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>El titular indica que la Asamblea está debatiendo la renovación del contrato de Ciudad del Saber y que existen cuestionamientos por exoneraciones.</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>[N-5bf4576df900:titulo] "Asamblea: Debate por la renovación del contrato de Ciudad del Saber genera cuestionamientos por exoneraciones"</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una opción del menú desplegable." type="list">
+      <formula1>"si,parcial,no"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fichas: citar medio y unidad cuando se nombran, y bloquear fichas sin afirmaciones
</commit_message>
<xml_diff>
--- a/backend/eval/planilla_etiquetas.xlsx
+++ b/backend/eval/planilla_etiquetas.xlsx
@@ -5254,7 +5254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5319,13 +5319,14 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Mitradel publico nuevas vacantes de empleo en su portal, segun reporto TVN el 7 de octubre de 2026.</t>
+          <t>TVN publicó con fecha 2026-10-07T21:34:03Z una noticia titulada "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles".</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"
-[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"</t>
+          <t>[N-6ffd1c40b65f:medio] "TVN"
+[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
         </is>
       </c>
       <c r="F2" s="7" t="n"/>
@@ -5347,13 +5348,14 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>La tasa de desempleo anual en Panama para el ano 2024 fue de 8.451% de la poblacion activa.</t>
+          <t>El dato anual histórico de desempleo registrado por el Banco Mundial para Panamá en el año 2024 fue de 8.451 % de la población activa.</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
-[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024</t>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:unidad] "% de la población activa"</t>
         </is>
       </c>
       <c r="F3" s="7" t="n"/>
@@ -5370,17 +5372,19 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>afirmación (hecho)</t>
+          <t>brief</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>En 2023, la tasa de desempleo registrada en Panama fue de 6.544%.</t>
+          <t>El medio TVN [N-6ffd1c40b65f:medio] publicó el 2026-10-07T21:34:03Z [N-6ffd1c40b65f:fecha] un reporte titulado "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles" [N-6ffd1c40b65f:titulo].</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+          <t>[N-6ffd1c40b65f:medio] "TVN"
+[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
         </is>
       </c>
       <c r="F4" s="7" t="n"/>
@@ -5402,13 +5406,14 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>El medio TVN publico el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] que Mitradel habilito nuevas vacantes de empleo en su portal web [N-6ffd1c40b65f:titulo].</t>
+          <t>Como contexto histórico de referencia previa, el indicador anual del Banco Mundial situó el desempleo en Panamá para el año 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] en 8.451 [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] % de la población activa [WB:PAN:SL.UEM.TOTL.ZS:2024:unidad].</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
-[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:unidad] "% de la población activa"</t>
         </is>
       </c>
       <c r="F5" s="7" t="n"/>
@@ -5425,20 +5430,19 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>brief</t>
+          <t>guion_45_60s</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Por otro lado, los datos historicos del Banco Mundial indican que en el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] la tasa de desempleo en Panama fue de 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa, mostrando un incremento en comparacion con el 6.544% [WB:PAN:SL.UEM.TOTL.ZS:2024:serie] registrado en el ano 2023 [WB:PAN:SL.UEM.TOTL.ZS:2024:serie].</t>
+          <t>El medio TVN [N-6ffd1c40b65f:medio] publicó el 2026-10-07T21:34:03Z [N-6ffd1c40b65f:fecha] una información titulada "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles" [N-6ffd1c40b65f:titulo].</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
-[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
-[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]
-[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+          <t>[N-6ffd1c40b65f:medio] "TVN"
+[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
         </is>
       </c>
       <c r="F6" s="7" t="n"/>
@@ -5455,19 +5459,19 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>brief</t>
+          <t>guion_45_60s</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>En la region, para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio], Costa Rica registro 6.936% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] y Republica Dominicana 5.312% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion].</t>
+          <t>Como antecedente histórico del mercado laboral, el Banco Mundial registró para Panamá en el año 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] una tasa de desempleo de 8.451 [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] % de la población activa [WB:PAN:SL.UEM.TOTL.ZS:2024:unidad].</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
           <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
-[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]
-[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]</t>
+[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:unidad] "% de la población activa"</t>
         </is>
       </c>
       <c r="F7" s="7" t="n"/>
@@ -5484,17 +5488,18 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>guion_45_60s</t>
+          <t>copy_digital</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>El medio TVN informo el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] sobre la publicacion de nuevas vacantes de empleo en el portal de Mitradel [N-6ffd1c40b65f:titulo].</t>
+          <t>TVN [N-6ffd1c40b65f:medio] publicó el 2026-10-07T21:34:03Z [N-6ffd1c40b65f:fecha] que el Mitradel habilitó nuevas vacantes laborales en su portal web [N-6ffd1c40b65f:titulo].</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
+          <t>[N-6ffd1c40b65f:medio] "TVN"
+[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
 [N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
         </is>
       </c>
@@ -5512,18 +5517,19 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>guion_45_60s</t>
+          <t>copy_digital</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Esta iniciativa surge en un contexto donde, segun datos historicos del Banco Mundial, la tasa de desempleo en Panama para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] se situo en 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa.</t>
+          <t>Como referencia histórica previa, el Banco Mundial situó el desempleo en Panamá en 8.451 [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] % de la población activa [WB:PAN:SL.UEM.TOTL.ZS:2024:unidad] en el año 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio].</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
-[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451</t>
+          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
+[WB:PAN:SL.UEM.TOTL.ZS:2024:unidad] "% de la población activa"
+[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024</t>
         </is>
       </c>
       <c r="F9" s="7" t="n"/>
@@ -5535,23 +5541,24 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-6ffd1c40b65f</t>
+          <t>CASO-EV-N-3d58bd578f4b</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>guion_45_60s</t>
+          <t>afirmación (declaracion)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Esta cifra represento un aumento frente al 6.544% [WB:PAN:SL.UEM.TOTL.ZS:2024:serie] reportado en el ano 2023 [WB:PAN:SL.UEM.TOTL.ZS:2024:serie].</t>
+          <t>El medio TVN publico el 8 de octubre de 2026 una noticia cuyo titular indica que mas de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]
-[WB:PAN:SL.UEM.TOTL.ZS:2024:serie] [{"anio": 2020, "valor": 14.663}, {"anio": 2021, "valor": 10.177}, {"anio": 2022, "valor": 8.086}, {"anio": 2023, "valor": 6.544}, {"anio": 2024, "valor": 8.451}]</t>
+          <t>[N-3d58bd578f4b:medio] "TVN"
+[N-3d58bd578f4b:fecha] "2026-10-08T18:27:29Z"
+[N-3d58bd578f4b:titulo] "Más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas"</t>
         </is>
       </c>
       <c r="F10" s="7" t="n"/>
@@ -5563,24 +5570,24 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-6ffd1c40b65f</t>
+          <t>CASO-EV-N-1a8d986bf866</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>guion_45_60s</t>
+          <t>afirmación (declaracion)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>En la comparacion regional del ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio], Costa Rica registro un desempleo de 6.936% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] y Republica Dominicana un 5.312% [WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion].</t>
+          <t>El titular indica una explosión demográfica en Panamá Este que aumenta la presión sobre el transporte público.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
-[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]
-[WB:PAN:SL.UEM.TOTL.ZS:2024:comparacion] [{"pais": "CRI", "anio": 2024, "valor": 6.936}, {"pais": "DOM", "anio": 2024, "valor": 5.312}]</t>
+          <t>[N-1a8d986bf866:titulo] "Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público"
+[N-1a8d986bf866:medio] "TVN"
+[N-1a8d986bf866:fecha] "2026-10-08T12:55:10Z"</t>
         </is>
       </c>
       <c r="F11" s="7" t="n"/>
@@ -5592,23 +5599,24 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-6ffd1c40b65f</t>
+          <t>CASO-EV-N-e2e7ae51395c</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>copy_digital</t>
+          <t>afirmación (declaracion)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Mitradel publica nuevas vacantes de empleo en su portal web, segun reporto TVN el 7 de octubre de 2026 [N-6ffd1c40b65f:fecha] [N-6ffd1c40b65f:titulo].</t>
+          <t>Según TVN, el ITSE se suma a una iniciativa para proyectar el café panameño y formar baristas.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>[N-6ffd1c40b65f:fecha] "2026-10-07T21:34:03Z"
-[N-6ffd1c40b65f:titulo] "Empleos en Panamá: Mitradel publica en su portal nuevas vacantes disponibles"</t>
+          <t>[N-e2e7ae51395c:titulo] "ITSE se suma a iniciativa para proyectar el café panameño y formar baristas"
+[N-e2e7ae51395c:medio] "TVN"
+[N-e2e7ae51395c:fecha] "2026-10-07T22:55:56Z"</t>
         </is>
       </c>
       <c r="F12" s="7" t="n"/>
@@ -5620,24 +5628,24 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-6ffd1c40b65f</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>copy_digital</t>
+          <t>afirmación (declaracion)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Como contexto historico, la tasa de desempleo en Panama para el ano 2024 [WB:PAN:SL.UEM.TOTL.ZS:2024:anio] fue de 8.451% [WB:PAN:SL.UEM.TOTL.ZS:2024:valor] de la poblacion activa, segun registros del Banco Mundial [WB:PAN:SL.UEM.TOTL.ZS:2024:valor].</t>
+          <t>El FMI proyecta que la economía de Panamá crecerá cerca de 5% en 2026.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>[WB:PAN:SL.UEM.TOTL.ZS:2024:anio] 2024
-[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451
-[WB:PAN:SL.UEM.TOTL.ZS:2024:valor] 8.451</t>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-34877dd09e6b:medio] "TVN"
+[N-34877dd09e6b:fecha] "2026-10-07T22:00:00Z"</t>
         </is>
       </c>
       <c r="F13" s="7" t="n"/>
@@ -5649,7 +5657,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-3d58bd578f4b</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5659,13 +5667,14 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Según un titular publicado por el medio TVN el 8 de octubre de 2026, más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas.</t>
+          <t>Un economista explicará el impacto de las tasas de interés en la economía panameña y la posible subida de cuotas de préstamos.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>[N-3d58bd578f4b:titulo] "Más de 200 universitarios participan en la Hackathon Copa Airlines 2026 en Veraguas"
-[N-3d58bd578f4b:fecha] "2026-10-08T18:27:29Z"</t>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"
+[N-bc0c4a46f2c5:medio] "TVN"
+[N-bc0c4a46f2c5:fecha] "2026-10-08T13:23:50Z"</t>
         </is>
       </c>
       <c r="F14" s="7" t="n"/>
@@ -5677,22 +5686,24 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-33f2663b5f67</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>afirmación (declaracion)</t>
+          <t>brief</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>El titular informa que el MOP avanza en más del 45% una nueva ruta para desahogar la vía Interamericana en David.</t>
+          <t>TVN informó que el FMI proyecta un crecimiento cercano al 5% para la economía de Panamá en 2026 [N-34877dd09e6b:titulo][N-34877dd09e6b:medio][N-34877dd09e6b:fecha].</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>[N-33f2663b5f67:titulo] "MOP avanza en mas del 45% nueva ruta para desahogar la via Interamericana en David"</t>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-34877dd09e6b:medio] "TVN"
+[N-34877dd09e6b:fecha] "2026-10-07T22:00:00Z"</t>
         </is>
       </c>
       <c r="F15" s="7" t="n"/>
@@ -5704,22 +5715,24 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-7f5a31e89279</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>afirmación (declaracion)</t>
+          <t>brief</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>TVN reporta que en Bocas del Toro se están afinando los detalles para el III Simulacro de Evacuación.</t>
+          <t>Además, otro titular indica que un economista explicará cómo las tasas de interés podrían elevar las cuotas de préstamos en el país [N-bc0c4a46f2c5:titulo][N-bc0c4a46f2c5:medio][N-bc0c4a46f2c5:fecha].</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>[N-7f5a31e89279:titulo] "Bocas del Toro afina detalles para el III Simulacro de Evacuación este lunes 12 de octubre"</t>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"
+[N-bc0c4a46f2c5:medio] "TVN"
+[N-bc0c4a46f2c5:fecha] "2026-10-08T13:23:50Z"</t>
         </is>
       </c>
       <c r="F16" s="7" t="n"/>
@@ -5731,22 +5744,23 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-7f5a31e89279</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>afirmación (declaracion)</t>
+          <t>guion_45_60s</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>El simulacro está programado para el lunes 12 de octubre.</t>
+          <t>El primero señala que el Fondo Monetario Internacional proyecta un crecimiento cercano al cinco por ciento para el año 2026 [N-34877dd09e6b:titulo][N-34877dd09e6b:fecha].</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>[N-7f5a31e89279:titulo] "Bocas del Toro afina detalles para el III Simulacro de Evacuación este lunes 12 de octubre"</t>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-34877dd09e6b:fecha] "2026-10-07T22:00:00Z"</t>
         </is>
       </c>
       <c r="F17" s="7" t="n"/>
@@ -5758,22 +5772,23 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-c4339fd4cfad</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>afirmación (declaracion)</t>
+          <t>guion_45_60s</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>El proyecto modificado plantea 30% menos en compra de pañales, telefonía y otros beneficios para jubilados.</t>
+          <t>El segundo anuncia que un economista explicará cómo las tasas de interés podrían elevar las cuotas de los préstamos en el país [N-bc0c4a46f2c5:titulo][N-bc0c4a46f2c5:fecha].</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>[N-c4339fd4cfad:titulo] "Descuentos para jubilados: Proyecto modificado plantea 30% menos en compra de pañales, telefonía y otros beneficios"</t>
+          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"
+[N-bc0c4a46f2c5:fecha] "2026-10-08T13:23:50Z"</t>
         </is>
       </c>
       <c r="F18" s="7" t="n"/>
@@ -5785,22 +5800,23 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-1a8d986bf866</t>
+          <t>CASO-EV-N-34877dd09e6b</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>afirmación (declaracion)</t>
+          <t>copy_digital</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público</t>
+          <t>TVN reporta que el FMI prevé un crecimiento del 5% para Panamá en 2026 y que un economista analizará el posible aumento de cuotas de préstamos por las tasas de interés [N-34877dd09e6b:titulo][N-bc0c4a46f2c5:titulo].</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>[N-1a8d986bf866:titulo] "Explosión demográfica en Panamá Este aumenta la presión sobre el transporte público"</t>
+          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
+[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
         </is>
       </c>
       <c r="F19" s="7" t="n"/>
@@ -5812,7 +5828,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-e2e7ae51395c</t>
+          <t>CASO-EV-N-e7673d45b48a</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -5822,12 +5838,14 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>El ITSE se incorpora a una iniciativa que busca proyectar el café panameño y capacitar baristas.</t>
+          <t>Lau Cortés: Ordenan detención domiciliaria e imputan cargos por enriquecimiento injustificado y blanqueo de capitales</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>[N-e2e7ae51395c:titulo] "ITSE se suma a iniciativa para proyectar el café panameño y formar baristas"</t>
+          <t>[N-e7673d45b48a:titulo] "Lau Cortés: Ordenan detención domiciliaria e imputan cargos por enriquecimiento injustificado y blanqueo de capitales"
+[N-e7673d45b48a:medio] "TVN"
+[N-e7673d45b48a:fecha] "2026-10-08T02:30:00Z"</t>
         </is>
       </c>
       <c r="F20" s="7" t="n"/>
@@ -5839,7 +5857,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
+          <t>CASO-EV-N-5bf4576df900</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -5849,293 +5867,22 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>TVN publicó un titular que indica que el FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026.</t>
+          <t>La Asamblea debatió la renovación del contrato de Ciudad del Saber, generando cuestionamientos por exoneraciones.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
-[N-34877dd09e6b:medio] "TVN"</t>
+          <t>[N-5bf4576df900:titulo] "Asamblea: Debate por la renovación del contrato de Ciudad del Saber genera cuestionamientos por exoneraciones"
+[N-5bf4576df900:medio] "TVN"
+[N-5bf4576df900:fecha] "2026-10-08T01:14:47Z"</t>
         </is>
       </c>
       <c r="F21" s="7" t="n"/>
       <c r="G21" s="7" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="6" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>afirmación (declaracion)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>TVN publicó un titular que pregunta si subirán las cuotas de préstamos y menciona que un economista explica el impacto de las tasas de interés en la economía panameña.</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"
-[N-bc0c4a46f2c5:medio] "TVN"</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>brief</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>TVN publicó un titular indicando que el FMI proyecta un crecimiento cercano al 5% para la economía de Panamá en 2026 [N-34877dd09e6b:titulo].</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>brief</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>En otra publicación, el medio plantea la pregunta sobre si subirán las cuotas de préstamos, citando a un economista que explica el impacto de las tasas de interés [N-bc0c4a46f2c5:titulo].</t>
-        </is>
-      </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>guion_45_60s</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>El primero indica que el FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026 [N-34877dd09e6b:titulo].</t>
-        </is>
-      </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>guion_45_60s</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Esta información fue publicada por el medio el 7 de octubre de 2026 [N-34877dd09e6b:fecha].</t>
-        </is>
-      </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>[N-34877dd09e6b:fecha] "2026-10-07T22:00:00Z"</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>guion_45_60s</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>En una segunda nota, TVN pregunta si subirán las cuotas de préstamos, mencionando que un economista explica el impacto de las tasas de interés en la economía panameña [N-bc0c4a46f2c5:titulo].</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>guion_45_60s</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Esta publicación data del 8 de octubre de 2026 [N-bc0c4a46f2c5:fecha].</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>[N-bc0c4a46f2c5:fecha] "2026-10-08T13:23:50Z"</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-34877dd09e6b</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>copy_digital</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>TVN reporta que el FMI proyecta un crecimiento cercano al 5% para 2026 [N-34877dd09e6b:titulo] y debate el impacto de las tasas de interés en las cuotas de préstamos [N-bc0c4a46f2c5:titulo].</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>[N-34877dd09e6b:titulo] "FMI proyecta que la economía de Panamá crecerá cerca de 5% este 2026"
-[N-bc0c4a46f2c5:titulo] "¿Subirán las cuotas de préstamos? Economista explica el impacto de las tasas de interés en la economía panameña"</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-e7673d45b48a</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>afirmación (declaracion)</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>TVN informa que se ordenó la detención domiciliaria e imputaron cargos a Lau Cortés por enriquecimiento injustificado y blanqueo de capitales.</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>[N-e7673d45b48a:titulo] "Lau Cortés: Ordenan detención domiciliaria e imputan cargos por enriquecimiento injustificado y blanqueo de capitales"</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>CASO-EV-N-5bf4576df900</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>afirmación (declaracion)</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>El titular indica que la Asamblea está debatiendo la renovación del contrato de Ciudad del Saber y que existen cuestionamientos por exoneraciones.</t>
-        </is>
-      </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>[N-5bf4576df900:titulo] "Asamblea: Debate por la renovación del contrato de Ciudad del Saber genera cuestionamientos por exoneraciones"</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una opción del menú desplegable." type="list">
+    <dataValidation sqref="F2:F21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="Elija una opción del menú desplegable." type="list">
       <formula1>"si,parcial,no"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>